<commit_message>
Export LMB : catalogue LMB complet (actifs + archivés), statut de l'article LMB par produit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/export-lmb/refs-lmb-manquantes.xlsx
+++ b/abc-terroirs/export-lmb/refs-lmb-manquantes.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sans réf. LMB" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Réf. à vérifier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En ligne mais archivés LMB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sans réf. LMB'!$A$1:$H$10</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +43,15 @@
     <font>
       <name val="Arial"/>
       <color rgb="00888888"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -75,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -104,6 +114,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2190,4 +2204,767 @@
   <autoFilter ref="A1:I36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Désignation (site)</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Prix TTC site (€)</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Réf. LMB</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Libellé LMB</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>À faire</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>ID PrestaShop</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>Lien produit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Whisky Hellyers Road – Tasmanie</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>A-02604</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>WHISKY HELLYERS ROAD  (Tasmanie)</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="11" t="n">
+        <v>116</v>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=116&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Tête de Lard (cabernet franc) – Manoir de la Tête Rouge</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>A-01760</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>TÊTE DE LARD (Cab franc) - Manoir de la Tête Rouge</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n"/>
+      <c r="F3" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=143&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Muscadet en biodynamie – Domaine de la Pépière</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>A-01300</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>MUSCADET - LA PEPIERE</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="n"/>
+      <c r="F4" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=165&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Amandes caramélisées bio 110 g</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>A-00289</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>AMANDES CARAMÉLISEÉS BIO 110g</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="11" t="n">
+        <v>199</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=199&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Rhum Fontanel blanc – Rhumerie du Vignoble</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>A-04087</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>RHUM FONTANEL BLANC - RHUMERIE DU VIGNOBLE</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="11" t="n">
+        <v>258</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=258&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Gin Sakurao Original – Japon</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>A-03733</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>GIN SAKURAO ORIGINAL - Japon</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="11" t="n">
+        <v>300</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=300&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Demi-mètre de bières nantaises</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>A-00770</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>DEMI MÈTRE BIÈRES NANTAISES</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="11" t="n">
+        <v>311</v>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=311&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Whisky Teeling Single Grain – Irlande</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>A-03626</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>WHISKY TEELING Single Grain (non tourbé) - IRLANDE</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="11" t="n">
+        <v>339</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=339&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Gin Ki No Bi – Japon</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>A-04732</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>GIN KI NO BI CLASSIC (eucalyptus, florale) - JAPON</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="11" t="n">
+        <v>348</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=348&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Rhum La Perle – A1710</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>A-05140</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>RHUM BLANC LA PERLE - A1710</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="11" t="n">
+        <v>384</v>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=384&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Coffret Voyage extraordinaire – Petit</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>A-05220</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>COFFRET VOYAGE EXTRAORDINAIRE V1</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="11" t="n">
+        <v>390</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=390&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Diablotine petite 37,5 cl</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>A-00782</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>DIABLOTINE PETITE 37.5cl</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="11" t="n">
+        <v>467</v>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=467&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>La Petite Menthe – Brasserie La Hulotte</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>A-05219</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>LIQUEUR PETITE MENTHE - LA HULOTTE</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="11" t="n">
+        <v>468</v>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=468&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Boîte savon Tour LU noir et blanc petits beurres 28 g</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>A-05421</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>PBB BOITE SAVON TOUR LU N&amp;B PETIT BEURRE 35g</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="11" t="n">
+        <v>481</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=481&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Boîte Délices &amp; Gourmandises sucrée-salée</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>A-05653</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>BOITE DELICES ET GOURMANDISES sucrée salée Be happy Sweet Home</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="11" t="n">
+        <v>503</v>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=503&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Whisky Porh Puce – Kaerilis 50 cl</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>A-04255</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>WHISKY PORH PUCE Kaerilis 50cl</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="11" t="n">
+        <v>508</v>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=508&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Gin Etsu Pacific Ocean Water – Distillerie Asahikawa, Japon 20 cl</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>A-05713</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>GIN ETSU OCEAN WATER 20CL</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="11" t="n">
+        <v>529</v>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=529&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Gin Saxon Garden – Wessex</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>A-04437</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>GIN SAXON GARDEN (florale, pure, élégant) - Angleterre</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="11" t="n">
+        <v>532</v>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=532&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Gâteau nantais, boîte de 2 bouchées 40 g</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>A-00940</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>GN GATEAU NANTAIS BOUCHÉES X2 40g</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="11" t="n">
+        <v>619</v>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=619&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Rhum Clairin Casimir – Haïti (en rupture)</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>A-04671</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>RHUM CLAIRIN CASIMIR - Haiti</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="11" t="n">
+        <v>622</v>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=622&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Coffret petit beurre « Bonnes fêtes » sucré-salé – Petit</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>A-06349</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>BOITE PB PETIT BEURRE NANTES V1</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=650&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Boîte petits beurres « Bonnes fêtes »</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>A-03183</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>BOITE BONNE FETES V2</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="11" t="n">
+        <v>671</v>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=671&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Fondant baulois, boîte de 2 bouchées</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>A-00110</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>FB FONDANT BAULOIS boite 2 BOUCHEES</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="11" t="n">
+        <v>707</v>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=707&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Sardines à poêler au beurre de baratte – La Perle des Dieux</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>A-01636</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>SARDINES AU BEURRE BARATTE A POELER 115g Perle des Dieux</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="11" t="n">
+        <v>711</v>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>https://abcterroirs.com/index.php?id_product=711&amp;controller=product</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Produits en vente sur le site dont l'article LMB est archivé. Colonne « À faire » : désactiver sur le site, ou réactiver dans LMB.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>